<commit_message>
Finishing adding 320 MHz clocks
</commit_message>
<xml_diff>
--- a/ClockBuilderPRO/projects/ConfigurationIndex.xlsx
+++ b/ClockBuilderPRO/projects/ConfigurationIndex.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\6089-127_CM_V3\GitHub\Cornell_CM_Rev3_HW\ClockBuilderPRO\projects\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\6089-127_CM_V3\GitHub\ClockBuilderPRO\projects\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF084C23-D8D5-48D5-85C4-DC92D7E5087E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A45E379-A6A4-46B7-8A99-0B536B5CC63C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{317829E7-0442-4B0F-847B-BF9A16B0382F}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="35">
   <si>
     <t>Out 1</t>
   </si>
@@ -134,6 +134,12 @@
   </si>
   <si>
     <t>Green cells indicate the input sources</t>
+  </si>
+  <si>
+    <t>R0Av3C02</t>
+  </si>
+  <si>
+    <t>R0Bv3C02</t>
   </si>
 </sst>
 </file>
@@ -610,7 +616,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AAA10E1-D638-4109-9638-B5E913BD74DD}">
-  <dimension ref="A1:S49"/>
+  <dimension ref="A1:S51"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13" style="1" customWidth="1"/>
@@ -782,81 +788,139 @@
       </c>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A12" s="7"/>
-      <c r="S12" s="8"/>
+      <c r="A12" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" s="9">
+        <v>48</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I12" s="1">
+        <v>320</v>
+      </c>
+      <c r="J12" s="1">
+        <v>320</v>
+      </c>
+      <c r="K12" s="1">
+        <v>320</v>
+      </c>
+      <c r="L12" s="1">
+        <v>320</v>
+      </c>
+      <c r="M12" s="1">
+        <v>320</v>
+      </c>
+      <c r="N12" s="1">
+        <v>320</v>
+      </c>
+      <c r="O12" s="1">
+        <v>320</v>
+      </c>
+      <c r="P12" s="1">
+        <v>320</v>
+      </c>
+      <c r="Q12" s="1">
+        <v>320</v>
+      </c>
+      <c r="R12" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="S12" s="8" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="7"/>
+      <c r="S13" s="8"/>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B14" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="9">
+      <c r="C14" s="9">
         <v>48</v>
       </c>
-      <c r="D13" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="H13" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="I13" s="1">
-        <v>322.265625</v>
-      </c>
-      <c r="J13" s="1">
-        <v>322.265625</v>
-      </c>
-      <c r="K13" s="1">
-        <v>322.265625</v>
-      </c>
-      <c r="L13" s="1">
-        <v>322.265625</v>
-      </c>
-      <c r="M13" s="1">
-        <v>322.265625</v>
-      </c>
-      <c r="N13" s="1">
-        <v>322.265625</v>
-      </c>
-      <c r="O13" s="1">
-        <v>322.265625</v>
-      </c>
-      <c r="P13" s="1">
-        <v>322.265625</v>
-      </c>
-      <c r="Q13" s="1">
-        <v>322.265625</v>
-      </c>
-      <c r="R13" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="S13" s="8" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A14" s="7"/>
-      <c r="S14" s="8"/>
+      <c r="D14" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I14" s="1">
+        <v>322.265625</v>
+      </c>
+      <c r="J14" s="1">
+        <v>322.265625</v>
+      </c>
+      <c r="K14" s="1">
+        <v>322.265625</v>
+      </c>
+      <c r="L14" s="1">
+        <v>322.265625</v>
+      </c>
+      <c r="M14" s="1">
+        <v>322.265625</v>
+      </c>
+      <c r="N14" s="1">
+        <v>322.265625</v>
+      </c>
+      <c r="O14" s="1">
+        <v>322.265625</v>
+      </c>
+      <c r="P14" s="1">
+        <v>322.265625</v>
+      </c>
+      <c r="Q14" s="1">
+        <v>322.265625</v>
+      </c>
+      <c r="R14" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="S14" s="8" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D15" s="9">
-        <v>320.64</v>
+      <c r="C15" s="9">
+        <v>48</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>18</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>18</v>
@@ -864,44 +928,44 @@
       <c r="F15" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G15" s="9">
-        <v>320.64</v>
-      </c>
-      <c r="H15" s="1">
-        <v>320.64</v>
+      <c r="G15" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>19</v>
       </c>
       <c r="I15" s="1">
-        <v>320.64</v>
+        <v>320</v>
       </c>
       <c r="J15" s="1">
-        <v>320.64</v>
+        <v>320</v>
       </c>
       <c r="K15" s="1">
-        <v>320.64</v>
+        <v>320</v>
       </c>
       <c r="L15" s="1">
-        <v>320.64</v>
+        <v>320</v>
       </c>
       <c r="M15" s="1">
-        <v>320.64</v>
+        <v>320</v>
       </c>
       <c r="N15" s="1">
-        <v>320.64</v>
+        <v>320</v>
       </c>
       <c r="O15" s="1">
-        <v>320.64</v>
+        <v>320</v>
       </c>
       <c r="P15" s="1">
-        <v>320.64</v>
+        <v>320</v>
       </c>
       <c r="Q15" s="1">
-        <v>320.64</v>
+        <v>320</v>
       </c>
       <c r="R15" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="S15" s="8">
-        <v>320.64</v>
+        <v>19</v>
+      </c>
+      <c r="S15" s="8" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.25">
@@ -910,22 +974,22 @@
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D17" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E17" s="9">
-        <v>40.08</v>
+      <c r="D17" s="9">
+        <v>320.64</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>18</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>18</v>
       </c>
       <c r="G17" s="9">
-        <v>40.08</v>
+        <v>320.64</v>
       </c>
       <c r="H17" s="1">
         <v>320.64</v>
@@ -957,11 +1021,11 @@
       <c r="Q17" s="1">
         <v>320.64</v>
       </c>
-      <c r="R17" s="1">
-        <v>40.08</v>
+      <c r="R17" s="1" t="s">
+        <v>18</v>
       </c>
       <c r="S17" s="8">
-        <v>40.08</v>
+        <v>320.64</v>
       </c>
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.25">
@@ -969,83 +1033,139 @@
       <c r="S18" s="8"/>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A19" s="10" t="s">
+      <c r="A19" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E19" s="9">
+        <v>40.08</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G19" s="9">
+        <v>40.08</v>
+      </c>
+      <c r="H19" s="1">
+        <v>320.64</v>
+      </c>
+      <c r="I19" s="1">
+        <v>320.64</v>
+      </c>
+      <c r="J19" s="1">
+        <v>320.64</v>
+      </c>
+      <c r="K19" s="1">
+        <v>320.64</v>
+      </c>
+      <c r="L19" s="1">
+        <v>320.64</v>
+      </c>
+      <c r="M19" s="1">
+        <v>320.64</v>
+      </c>
+      <c r="N19" s="1">
+        <v>320.64</v>
+      </c>
+      <c r="O19" s="1">
+        <v>320.64</v>
+      </c>
+      <c r="P19" s="1">
+        <v>320.64</v>
+      </c>
+      <c r="Q19" s="1">
+        <v>320.64</v>
+      </c>
+      <c r="R19" s="1">
+        <v>40.08</v>
+      </c>
+      <c r="S19" s="8">
+        <v>40.08</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A20" s="7"/>
+      <c r="E20" s="9"/>
+      <c r="G20" s="9"/>
+      <c r="S20" s="8"/>
+    </row>
+    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A21" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="B19" s="11" t="s">
+      <c r="B21" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="C19" s="11"/>
-      <c r="D19" s="12">
-        <v>320.64</v>
-      </c>
-      <c r="E19" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="F19" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="G19" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="H19" s="11">
-        <v>320.64</v>
-      </c>
-      <c r="I19" s="11">
-        <v>320.64</v>
-      </c>
-      <c r="J19" s="11">
-        <v>320.64</v>
-      </c>
-      <c r="K19" s="11">
-        <v>320.64</v>
-      </c>
-      <c r="L19" s="11">
-        <v>320.64</v>
-      </c>
-      <c r="M19" s="11">
-        <v>320.64</v>
-      </c>
-      <c r="N19" s="11">
-        <v>320.64</v>
-      </c>
-      <c r="O19" s="11">
-        <v>320.64</v>
-      </c>
-      <c r="P19" s="11">
-        <v>320.64</v>
-      </c>
-      <c r="Q19" s="11">
-        <v>320.64</v>
-      </c>
-      <c r="R19" s="11">
-        <v>320.64</v>
-      </c>
-      <c r="S19" s="13">
-        <v>320.64</v>
-      </c>
-    </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="S20" s="1"/>
-    </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="S21" s="1"/>
-    </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="S30" s="1"/>
-    </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="S31" s="1"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="12">
+        <v>320.64</v>
+      </c>
+      <c r="E21" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="F21" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G21" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="H21" s="11">
+        <v>320.64</v>
+      </c>
+      <c r="I21" s="11">
+        <v>320.64</v>
+      </c>
+      <c r="J21" s="11">
+        <v>320.64</v>
+      </c>
+      <c r="K21" s="11">
+        <v>320.64</v>
+      </c>
+      <c r="L21" s="11">
+        <v>320.64</v>
+      </c>
+      <c r="M21" s="11">
+        <v>320.64</v>
+      </c>
+      <c r="N21" s="11">
+        <v>320.64</v>
+      </c>
+      <c r="O21" s="11">
+        <v>320.64</v>
+      </c>
+      <c r="P21" s="11">
+        <v>320.64</v>
+      </c>
+      <c r="Q21" s="11">
+        <v>320.64</v>
+      </c>
+      <c r="R21" s="11">
+        <v>320.64</v>
+      </c>
+      <c r="S21" s="13">
+        <v>320.64</v>
+      </c>
+    </row>
+    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S22" s="1"/>
+    </row>
+    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S23" s="1"/>
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.25">
       <c r="S32" s="1"/>
     </row>
+    <row r="33" spans="19:19" x14ac:dyDescent="0.25">
+      <c r="S33" s="1"/>
+    </row>
     <row r="34" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S34" s="1"/>
     </row>
-    <row r="35" spans="19:19" x14ac:dyDescent="0.25">
-      <c r="S35" s="1"/>
-    </row>
     <row r="36" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S36" s="1"/>
     </row>
@@ -1055,12 +1175,12 @@
     <row r="38" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S38" s="1"/>
     </row>
+    <row r="39" spans="19:19" x14ac:dyDescent="0.25">
+      <c r="S39" s="1"/>
+    </row>
     <row r="40" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S40" s="1"/>
     </row>
-    <row r="41" spans="19:19" x14ac:dyDescent="0.25">
-      <c r="S41" s="1"/>
-    </row>
     <row r="42" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S42" s="1"/>
     </row>
@@ -1073,14 +1193,20 @@
     <row r="45" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S45" s="1"/>
     </row>
+    <row r="46" spans="19:19" x14ac:dyDescent="0.25">
+      <c r="S46" s="1"/>
+    </row>
     <row r="47" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S47" s="1"/>
     </row>
-    <row r="48" spans="19:19" x14ac:dyDescent="0.25">
-      <c r="S48" s="1"/>
-    </row>
     <row r="49" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S49" s="1"/>
+    </row>
+    <row r="50" spans="19:19" x14ac:dyDescent="0.25">
+      <c r="S50" s="1"/>
+    </row>
+    <row r="51" spans="19:19" x14ac:dyDescent="0.25">
+      <c r="S51" s="1"/>
     </row>
   </sheetData>
   <printOptions gridLines="1"/>

</xml_diff>